<commit_message>
Fix workbook drawdown seed to nominal projected portfolio; year cells as numbers
Co-authored-by: Festas <245144013+Festas@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/fire-simulator/public/templates/fire-analysis-template.xlsx
+++ b/fire-simulator/public/templates/fire-analysis-template.xlsx
@@ -1188,7 +1188,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
-        <f>1</f>
+        <v>1</v>
       </c>
       <c r="B2" s="8">
         <f>currentAge+1-1</f>
@@ -1223,7 +1223,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
-        <f>2</f>
+        <v>2</v>
       </c>
       <c r="B3" s="8">
         <f>currentAge+2-1</f>
@@ -1258,7 +1258,7 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
-        <f>3</f>
+        <v>3</v>
       </c>
       <c r="B4" s="8">
         <f>currentAge+3-1</f>
@@ -1293,7 +1293,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="8">
-        <f>4</f>
+        <v>4</v>
       </c>
       <c r="B5" s="8">
         <f>currentAge+4-1</f>
@@ -1328,7 +1328,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="8">
-        <f>5</f>
+        <v>5</v>
       </c>
       <c r="B6" s="8">
         <f>currentAge+5-1</f>
@@ -1363,7 +1363,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="8">
-        <f>6</f>
+        <v>6</v>
       </c>
       <c r="B7" s="8">
         <f>currentAge+6-1</f>
@@ -1398,7 +1398,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="8">
-        <f>7</f>
+        <v>7</v>
       </c>
       <c r="B8" s="8">
         <f>currentAge+7-1</f>
@@ -1433,7 +1433,7 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
-        <f>8</f>
+        <v>8</v>
       </c>
       <c r="B9" s="8">
         <f>currentAge+8-1</f>
@@ -1468,7 +1468,7 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="8">
-        <f>9</f>
+        <v>9</v>
       </c>
       <c r="B10" s="8">
         <f>currentAge+9-1</f>
@@ -1503,7 +1503,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
-        <f>10</f>
+        <v>10</v>
       </c>
       <c r="B11" s="8">
         <f>currentAge+10-1</f>
@@ -1538,7 +1538,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="8">
-        <f>11</f>
+        <v>11</v>
       </c>
       <c r="B12" s="8">
         <f>currentAge+11-1</f>
@@ -1573,7 +1573,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="8">
-        <f>12</f>
+        <v>12</v>
       </c>
       <c r="B13" s="8">
         <f>currentAge+12-1</f>
@@ -1608,7 +1608,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="8">
-        <f>13</f>
+        <v>13</v>
       </c>
       <c r="B14" s="8">
         <f>currentAge+13-1</f>
@@ -1643,7 +1643,7 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="8">
-        <f>14</f>
+        <v>14</v>
       </c>
       <c r="B15" s="8">
         <f>currentAge+14-1</f>
@@ -1678,7 +1678,7 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="8">
-        <f>15</f>
+        <v>15</v>
       </c>
       <c r="B16" s="8">
         <f>currentAge+15-1</f>
@@ -1713,7 +1713,7 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="8">
-        <f>16</f>
+        <v>16</v>
       </c>
       <c r="B17" s="8">
         <f>currentAge+16-1</f>
@@ -1748,7 +1748,7 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="8">
-        <f>17</f>
+        <v>17</v>
       </c>
       <c r="B18" s="8">
         <f>currentAge+17-1</f>
@@ -1783,7 +1783,7 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="8">
-        <f>18</f>
+        <v>18</v>
       </c>
       <c r="B19" s="8">
         <f>currentAge+18-1</f>
@@ -1818,7 +1818,7 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="8">
-        <f>19</f>
+        <v>19</v>
       </c>
       <c r="B20" s="8">
         <f>currentAge+19-1</f>
@@ -1853,7 +1853,7 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="8">
-        <f>20</f>
+        <v>20</v>
       </c>
       <c r="B21" s="8">
         <f>currentAge+20-1</f>
@@ -1888,7 +1888,7 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="8">
-        <f>21</f>
+        <v>21</v>
       </c>
       <c r="B22" s="8">
         <f>currentAge+21-1</f>
@@ -1923,7 +1923,7 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="8">
-        <f>22</f>
+        <v>22</v>
       </c>
       <c r="B23" s="8">
         <f>currentAge+22-1</f>
@@ -1958,7 +1958,7 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="8">
-        <f>23</f>
+        <v>23</v>
       </c>
       <c r="B24" s="8">
         <f>currentAge+23-1</f>
@@ -1993,7 +1993,7 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="8">
-        <f>24</f>
+        <v>24</v>
       </c>
       <c r="B25" s="8">
         <f>currentAge+24-1</f>
@@ -2028,7 +2028,7 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="8">
-        <f>25</f>
+        <v>25</v>
       </c>
       <c r="B26" s="8">
         <f>currentAge+25-1</f>
@@ -2063,7 +2063,7 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="8">
-        <f>26</f>
+        <v>26</v>
       </c>
       <c r="B27" s="8">
         <f>currentAge+26-1</f>
@@ -2098,7 +2098,7 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="8">
-        <f>27</f>
+        <v>27</v>
       </c>
       <c r="B28" s="8">
         <f>currentAge+27-1</f>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="8">
-        <f>28</f>
+        <v>28</v>
       </c>
       <c r="B29" s="8">
         <f>currentAge+28-1</f>
@@ -2168,7 +2168,7 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="8">
-        <f>29</f>
+        <v>29</v>
       </c>
       <c r="B30" s="8">
         <f>currentAge+29-1</f>
@@ -2203,7 +2203,7 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="8">
-        <f>30</f>
+        <v>30</v>
       </c>
       <c r="B31" s="8">
         <f>currentAge+30-1</f>
@@ -2238,7 +2238,7 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="8">
-        <f>31</f>
+        <v>31</v>
       </c>
       <c r="B32" s="8">
         <f>currentAge+31-1</f>
@@ -2273,7 +2273,7 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="8">
-        <f>32</f>
+        <v>32</v>
       </c>
       <c r="B33" s="8">
         <f>currentAge+32-1</f>
@@ -2308,7 +2308,7 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="8">
-        <f>33</f>
+        <v>33</v>
       </c>
       <c r="B34" s="8">
         <f>currentAge+33-1</f>
@@ -2343,7 +2343,7 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="8">
-        <f>34</f>
+        <v>34</v>
       </c>
       <c r="B35" s="8">
         <f>currentAge+34-1</f>
@@ -2378,7 +2378,7 @@
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="8">
-        <f>35</f>
+        <v>35</v>
       </c>
       <c r="B36" s="8">
         <f>currentAge+35-1</f>
@@ -2413,7 +2413,7 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="8">
-        <f>36</f>
+        <v>36</v>
       </c>
       <c r="B37" s="8">
         <f>currentAge+36-1</f>
@@ -2448,7 +2448,7 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="8">
-        <f>37</f>
+        <v>37</v>
       </c>
       <c r="B38" s="8">
         <f>currentAge+37-1</f>
@@ -2483,7 +2483,7 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="8">
-        <f>38</f>
+        <v>38</v>
       </c>
       <c r="B39" s="8">
         <f>currentAge+38-1</f>
@@ -2518,7 +2518,7 @@
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="8">
-        <f>39</f>
+        <v>39</v>
       </c>
       <c r="B40" s="8">
         <f>currentAge+39-1</f>
@@ -2553,7 +2553,7 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="8">
-        <f>40</f>
+        <v>40</v>
       </c>
       <c r="B41" s="8">
         <f>currentAge+40-1</f>
@@ -2588,7 +2588,7 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="8">
-        <f>41</f>
+        <v>41</v>
       </c>
       <c r="B42" s="8">
         <f>currentAge+41-1</f>
@@ -2623,7 +2623,7 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="8">
-        <f>42</f>
+        <v>42</v>
       </c>
       <c r="B43" s="8">
         <f>currentAge+42-1</f>
@@ -2658,7 +2658,7 @@
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="8">
-        <f>43</f>
+        <v>43</v>
       </c>
       <c r="B44" s="8">
         <f>currentAge+43-1</f>
@@ -2693,7 +2693,7 @@
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="8">
-        <f>44</f>
+        <v>44</v>
       </c>
       <c r="B45" s="8">
         <f>currentAge+44-1</f>
@@ -2728,7 +2728,7 @@
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="8">
-        <f>45</f>
+        <v>45</v>
       </c>
       <c r="B46" s="8">
         <f>currentAge+45-1</f>
@@ -2763,7 +2763,7 @@
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="8">
-        <f>46</f>
+        <v>46</v>
       </c>
       <c r="B47" s="8">
         <f>currentAge+46-1</f>
@@ -2798,7 +2798,7 @@
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="8">
-        <f>47</f>
+        <v>47</v>
       </c>
       <c r="B48" s="8">
         <f>currentAge+47-1</f>
@@ -2833,7 +2833,7 @@
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="8">
-        <f>48</f>
+        <v>48</v>
       </c>
       <c r="B49" s="8">
         <f>currentAge+48-1</f>
@@ -2868,7 +2868,7 @@
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="8">
-        <f>49</f>
+        <v>49</v>
       </c>
       <c r="B50" s="8">
         <f>currentAge+49-1</f>
@@ -2903,7 +2903,7 @@
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="8">
-        <f>50</f>
+        <v>50</v>
       </c>
       <c r="B51" s="8">
         <f>currentAge+50-1</f>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="8">
-        <f>51</f>
+        <v>51</v>
       </c>
       <c r="B52" s="8">
         <f>currentAge+51-1</f>
@@ -2973,7 +2973,7 @@
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="8">
-        <f>52</f>
+        <v>52</v>
       </c>
       <c r="B53" s="8">
         <f>currentAge+52-1</f>
@@ -3008,7 +3008,7 @@
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="8">
-        <f>53</f>
+        <v>53</v>
       </c>
       <c r="B54" s="8">
         <f>currentAge+53-1</f>
@@ -3043,7 +3043,7 @@
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="8">
-        <f>54</f>
+        <v>54</v>
       </c>
       <c r="B55" s="8">
         <f>currentAge+54-1</f>
@@ -3078,7 +3078,7 @@
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="8">
-        <f>55</f>
+        <v>55</v>
       </c>
       <c r="B56" s="8">
         <f>currentAge+55-1</f>
@@ -3113,7 +3113,7 @@
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="8">
-        <f>56</f>
+        <v>56</v>
       </c>
       <c r="B57" s="8">
         <f>currentAge+56-1</f>
@@ -3148,7 +3148,7 @@
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="8">
-        <f>57</f>
+        <v>57</v>
       </c>
       <c r="B58" s="8">
         <f>currentAge+57-1</f>
@@ -3183,7 +3183,7 @@
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="8">
-        <f>58</f>
+        <v>58</v>
       </c>
       <c r="B59" s="8">
         <f>currentAge+58-1</f>
@@ -3218,7 +3218,7 @@
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="8">
-        <f>59</f>
+        <v>59</v>
       </c>
       <c r="B60" s="8">
         <f>currentAge+59-1</f>
@@ -3253,7 +3253,7 @@
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="8">
-        <f>60</f>
+        <v>60</v>
       </c>
       <c r="B61" s="8">
         <f>currentAge+60-1</f>
@@ -3460,13 +3460,13 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
-        <f>1</f>
+        <v>1</v>
       </c>
       <c r="B2" s="8">
         <f>fireAge+1-1</f>
       </c>
       <c r="C2" s="9">
-        <f>'FIRE number'!B9</f>
+        <f>IFERROR(INDEX(Accumulation!$G:$G, MATCH(fireAge, Accumulation!$B:$B, 0)), 0)</f>
       </c>
       <c r="D2" s="9">
         <f>IF((fireAge+1-1) &lt;= endAge, MAX(0, (desiredIncome+healthMonthly)*12*(1+inflation/100)^((fireAge-currentAge)+1-1) - IF((fireAge+1-1)&gt;=pensionAge, statePension*12*(1+inflation/100)^((fireAge-currentAge)+1-1), 0)), 0)</f>
@@ -3486,7 +3486,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
-        <f>2</f>
+        <v>2</v>
       </c>
       <c r="B3" s="8">
         <f>fireAge+2-1</f>
@@ -3512,7 +3512,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
-        <f>3</f>
+        <v>3</v>
       </c>
       <c r="B4" s="8">
         <f>fireAge+3-1</f>
@@ -3538,7 +3538,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="8">
-        <f>4</f>
+        <v>4</v>
       </c>
       <c r="B5" s="8">
         <f>fireAge+4-1</f>
@@ -3564,7 +3564,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="8">
-        <f>5</f>
+        <v>5</v>
       </c>
       <c r="B6" s="8">
         <f>fireAge+5-1</f>
@@ -3590,7 +3590,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="8">
-        <f>6</f>
+        <v>6</v>
       </c>
       <c r="B7" s="8">
         <f>fireAge+6-1</f>
@@ -3616,7 +3616,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="8">
-        <f>7</f>
+        <v>7</v>
       </c>
       <c r="B8" s="8">
         <f>fireAge+7-1</f>
@@ -3642,7 +3642,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
-        <f>8</f>
+        <v>8</v>
       </c>
       <c r="B9" s="8">
         <f>fireAge+8-1</f>
@@ -3668,7 +3668,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="8">
-        <f>9</f>
+        <v>9</v>
       </c>
       <c r="B10" s="8">
         <f>fireAge+9-1</f>
@@ -3694,7 +3694,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
-        <f>10</f>
+        <v>10</v>
       </c>
       <c r="B11" s="8">
         <f>fireAge+10-1</f>
@@ -3720,7 +3720,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="8">
-        <f>11</f>
+        <v>11</v>
       </c>
       <c r="B12" s="8">
         <f>fireAge+11-1</f>
@@ -3746,7 +3746,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="8">
-        <f>12</f>
+        <v>12</v>
       </c>
       <c r="B13" s="8">
         <f>fireAge+12-1</f>
@@ -3772,7 +3772,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="8">
-        <f>13</f>
+        <v>13</v>
       </c>
       <c r="B14" s="8">
         <f>fireAge+13-1</f>
@@ -3798,7 +3798,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="8">
-        <f>14</f>
+        <v>14</v>
       </c>
       <c r="B15" s="8">
         <f>fireAge+14-1</f>
@@ -3824,7 +3824,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="8">
-        <f>15</f>
+        <v>15</v>
       </c>
       <c r="B16" s="8">
         <f>fireAge+15-1</f>
@@ -3850,7 +3850,7 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="8">
-        <f>16</f>
+        <v>16</v>
       </c>
       <c r="B17" s="8">
         <f>fireAge+16-1</f>
@@ -3876,7 +3876,7 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="8">
-        <f>17</f>
+        <v>17</v>
       </c>
       <c r="B18" s="8">
         <f>fireAge+17-1</f>
@@ -3902,7 +3902,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="8">
-        <f>18</f>
+        <v>18</v>
       </c>
       <c r="B19" s="8">
         <f>fireAge+18-1</f>
@@ -3928,7 +3928,7 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="8">
-        <f>19</f>
+        <v>19</v>
       </c>
       <c r="B20" s="8">
         <f>fireAge+19-1</f>
@@ -3954,7 +3954,7 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="8">
-        <f>20</f>
+        <v>20</v>
       </c>
       <c r="B21" s="8">
         <f>fireAge+20-1</f>
@@ -3980,7 +3980,7 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="8">
-        <f>21</f>
+        <v>21</v>
       </c>
       <c r="B22" s="8">
         <f>fireAge+21-1</f>
@@ -4006,7 +4006,7 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="8">
-        <f>22</f>
+        <v>22</v>
       </c>
       <c r="B23" s="8">
         <f>fireAge+22-1</f>
@@ -4032,7 +4032,7 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="8">
-        <f>23</f>
+        <v>23</v>
       </c>
       <c r="B24" s="8">
         <f>fireAge+23-1</f>
@@ -4058,7 +4058,7 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="8">
-        <f>24</f>
+        <v>24</v>
       </c>
       <c r="B25" s="8">
         <f>fireAge+24-1</f>
@@ -4084,7 +4084,7 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="8">
-        <f>25</f>
+        <v>25</v>
       </c>
       <c r="B26" s="8">
         <f>fireAge+25-1</f>
@@ -4110,7 +4110,7 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="8">
-        <f>26</f>
+        <v>26</v>
       </c>
       <c r="B27" s="8">
         <f>fireAge+26-1</f>
@@ -4136,7 +4136,7 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="8">
-        <f>27</f>
+        <v>27</v>
       </c>
       <c r="B28" s="8">
         <f>fireAge+27-1</f>
@@ -4162,7 +4162,7 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="8">
-        <f>28</f>
+        <v>28</v>
       </c>
       <c r="B29" s="8">
         <f>fireAge+28-1</f>
@@ -4188,7 +4188,7 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="8">
-        <f>29</f>
+        <v>29</v>
       </c>
       <c r="B30" s="8">
         <f>fireAge+29-1</f>
@@ -4214,7 +4214,7 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="8">
-        <f>30</f>
+        <v>30</v>
       </c>
       <c r="B31" s="8">
         <f>fireAge+30-1</f>
@@ -4240,7 +4240,7 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="8">
-        <f>31</f>
+        <v>31</v>
       </c>
       <c r="B32" s="8">
         <f>fireAge+31-1</f>
@@ -4266,7 +4266,7 @@
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="8">
-        <f>32</f>
+        <v>32</v>
       </c>
       <c r="B33" s="8">
         <f>fireAge+32-1</f>
@@ -4292,7 +4292,7 @@
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="8">
-        <f>33</f>
+        <v>33</v>
       </c>
       <c r="B34" s="8">
         <f>fireAge+33-1</f>
@@ -4318,7 +4318,7 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="8">
-        <f>34</f>
+        <v>34</v>
       </c>
       <c r="B35" s="8">
         <f>fireAge+34-1</f>
@@ -4344,7 +4344,7 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="8">
-        <f>35</f>
+        <v>35</v>
       </c>
       <c r="B36" s="8">
         <f>fireAge+35-1</f>
@@ -4370,7 +4370,7 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="8">
-        <f>36</f>
+        <v>36</v>
       </c>
       <c r="B37" s="8">
         <f>fireAge+36-1</f>
@@ -4396,7 +4396,7 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="8">
-        <f>37</f>
+        <v>37</v>
       </c>
       <c r="B38" s="8">
         <f>fireAge+37-1</f>
@@ -4422,7 +4422,7 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="8">
-        <f>38</f>
+        <v>38</v>
       </c>
       <c r="B39" s="8">
         <f>fireAge+38-1</f>
@@ -4448,7 +4448,7 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="8">
-        <f>39</f>
+        <v>39</v>
       </c>
       <c r="B40" s="8">
         <f>fireAge+39-1</f>
@@ -4474,7 +4474,7 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="8">
-        <f>40</f>
+        <v>40</v>
       </c>
       <c r="B41" s="8">
         <f>fireAge+40-1</f>
@@ -4500,7 +4500,7 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="8">
-        <f>41</f>
+        <v>41</v>
       </c>
       <c r="B42" s="8">
         <f>fireAge+41-1</f>
@@ -4526,7 +4526,7 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="8">
-        <f>42</f>
+        <v>42</v>
       </c>
       <c r="B43" s="8">
         <f>fireAge+42-1</f>
@@ -4552,7 +4552,7 @@
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="8">
-        <f>43</f>
+        <v>43</v>
       </c>
       <c r="B44" s="8">
         <f>fireAge+43-1</f>
@@ -4578,7 +4578,7 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="8">
-        <f>44</f>
+        <v>44</v>
       </c>
       <c r="B45" s="8">
         <f>fireAge+44-1</f>
@@ -4604,7 +4604,7 @@
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="8">
-        <f>45</f>
+        <v>45</v>
       </c>
       <c r="B46" s="8">
         <f>fireAge+45-1</f>
@@ -4630,7 +4630,7 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="8">
-        <f>46</f>
+        <v>46</v>
       </c>
       <c r="B47" s="8">
         <f>fireAge+46-1</f>
@@ -4656,7 +4656,7 @@
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="8">
-        <f>47</f>
+        <v>47</v>
       </c>
       <c r="B48" s="8">
         <f>fireAge+47-1</f>
@@ -4682,7 +4682,7 @@
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="8">
-        <f>48</f>
+        <v>48</v>
       </c>
       <c r="B49" s="8">
         <f>fireAge+48-1</f>
@@ -4708,7 +4708,7 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="8">
-        <f>49</f>
+        <v>49</v>
       </c>
       <c r="B50" s="8">
         <f>fireAge+49-1</f>
@@ -4734,7 +4734,7 @@
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="8">
-        <f>50</f>
+        <v>50</v>
       </c>
       <c r="B51" s="8">
         <f>fireAge+50-1</f>
@@ -4760,7 +4760,7 @@
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="8">
-        <f>51</f>
+        <v>51</v>
       </c>
       <c r="B52" s="8">
         <f>fireAge+51-1</f>
@@ -4786,7 +4786,7 @@
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="8">
-        <f>52</f>
+        <v>52</v>
       </c>
       <c r="B53" s="8">
         <f>fireAge+52-1</f>
@@ -4812,7 +4812,7 @@
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="8">
-        <f>53</f>
+        <v>53</v>
       </c>
       <c r="B54" s="8">
         <f>fireAge+53-1</f>
@@ -4838,7 +4838,7 @@
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="8">
-        <f>54</f>
+        <v>54</v>
       </c>
       <c r="B55" s="8">
         <f>fireAge+54-1</f>
@@ -4864,7 +4864,7 @@
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="8">
-        <f>55</f>
+        <v>55</v>
       </c>
       <c r="B56" s="8">
         <f>fireAge+55-1</f>
@@ -4890,7 +4890,7 @@
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="8">
-        <f>56</f>
+        <v>56</v>
       </c>
       <c r="B57" s="8">
         <f>fireAge+56-1</f>
@@ -4916,7 +4916,7 @@
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="8">
-        <f>57</f>
+        <v>57</v>
       </c>
       <c r="B58" s="8">
         <f>fireAge+57-1</f>
@@ -4942,7 +4942,7 @@
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="8">
-        <f>58</f>
+        <v>58</v>
       </c>
       <c r="B59" s="8">
         <f>fireAge+58-1</f>
@@ -4968,7 +4968,7 @@
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="8">
-        <f>59</f>
+        <v>59</v>
       </c>
       <c r="B60" s="8">
         <f>fireAge+59-1</f>
@@ -4994,7 +4994,7 @@
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="8">
-        <f>60</f>
+        <v>60</v>
       </c>
       <c r="B61" s="8">
         <f>fireAge+60-1</f>

</xml_diff>